<commit_message>
Add mount_offset to the master template; drop generated build outputs
* examples/Master_Template.xlsx regenerated with the new 'mount_offset'
  column (per-stiffener cross-aisle CG gap to the upright).
* examples/Master_Template_FINAL_mount_offset.xlsx: the provided master
  with the mount_offset column added and stiffener rows pre-filled with
  estimates (a header comment documents how to compute the exact value).
* Remove tracked generated outputs (out_rfem/, out_spr/ reports and
  images) and ignore those output directories - they are regenerated by
  the CLI and do not belong in the build.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QfGuquQv5GMUr3ffngBYoB
</commit_message>
<xml_diff>
--- a/examples/Master_Template.xlsx
+++ b/examples/Master_Template.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -530,24 +530,45 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mount_offset (stiffener rows only): cross-aisle distance from the upright</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BEAM_STIFFNESS: add a 'Kb @ UPL x.x' column per upright wall thickness; the</t>
+          <t>centroid line to the stiffener centroid line when mounted; the builder uses</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>it to place the stiffener node (else the app's global stiffener offset).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BEAM_STIFFNESS: add a 'Kb @ UPL x.x' column per upright wall thickness; the</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>beam connector stiffness is then chosen by the upright the beam bolts to.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>A company name is requested on import (sections are company-specific).</t>
         </is>
@@ -564,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -582,15 +603,16 @@
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="31" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="23" customWidth="1" min="23" max="23"/>
-    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="23" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -671,45 +693,50 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>mount_offset (mm) [stiffener centroid gap to upright]</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>depth_h (mm)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>width_b (mm)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>t (mm)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>e1 (mm)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>e2 (mm)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>curve_y</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>curve_z</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>connector_k (kNm/rad)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>connector_m_rd (kNm)</t>
         </is>
@@ -767,33 +794,34 @@
       <c r="O2" t="n">
         <v>4.59</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="n">
         <v>90</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>61</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>1.6</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>13.48</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>12.39</v>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -847,31 +875,32 @@
       <c r="O3" t="n">
         <v>0</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="n">
         <v>60</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>40</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>1.6</v>
       </c>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>200</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>1.14</v>
       </c>
     </row>
@@ -927,29 +956,30 @@
       <c r="O4" t="n">
         <v>0</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="n">
         <v>36</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>21</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>1.5</v>
       </c>
-      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1004,28 +1034,31 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q5" t="n">
         <v>159</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>128</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>2.5</v>
       </c>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>